<commit_message>
[portal] charge RR2401024582 · 2026-05-21 14:25
</commit_message>
<xml_diff>
--- a/Master-Data.xlsx
+++ b/Master-Data.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F833"/>
+  <dimension ref="A1:F834"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20419,14 +20419,42 @@
           <t>19/05/2026</t>
         </is>
       </c>
-      <c r="E833" t="inlineStr">
-        <is>
-          <t>27.555435</t>
-        </is>
-      </c>
-      <c r="F833" t="inlineStr">
-        <is>
-          <t>80.696812</t>
+      <c r="E833" t="n">
+        <v>27.555435</v>
+      </c>
+      <c r="F833" t="n">
+        <v>80.69681199999999</v>
+      </c>
+    </row>
+    <row r="834">
+      <c r="A834" t="inlineStr">
+        <is>
+          <t>RR2401024582</t>
+        </is>
+      </c>
+      <c r="B834" t="inlineStr">
+        <is>
+          <t>Reshma</t>
+        </is>
+      </c>
+      <c r="C834" t="inlineStr">
+        <is>
+          <t>8175011718</t>
+        </is>
+      </c>
+      <c r="D834" t="inlineStr">
+        <is>
+          <t>15/05/2026</t>
+        </is>
+      </c>
+      <c r="E834" t="inlineStr">
+        <is>
+          <t>27.5745</t>
+        </is>
+      </c>
+      <c r="F834" t="inlineStr">
+        <is>
+          <t>80.6951</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
[portal] charge RR2401024654 · 2026-05-21 14:27
</commit_message>
<xml_diff>
--- a/Master-Data.xlsx
+++ b/Master-Data.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F834"/>
+  <dimension ref="A1:F835"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20447,14 +20447,42 @@
           <t>15/05/2026</t>
         </is>
       </c>
-      <c r="E834" t="inlineStr">
-        <is>
-          <t>27.5745</t>
-        </is>
-      </c>
-      <c r="F834" t="inlineStr">
-        <is>
-          <t>80.6951</t>
+      <c r="E834" t="n">
+        <v>27.5745</v>
+      </c>
+      <c r="F834" t="n">
+        <v>80.6951</v>
+      </c>
+    </row>
+    <row r="835">
+      <c r="A835" t="inlineStr">
+        <is>
+          <t>RR2401024654</t>
+        </is>
+      </c>
+      <c r="B835" t="inlineStr">
+        <is>
+          <t>Naheem</t>
+        </is>
+      </c>
+      <c r="C835" t="inlineStr">
+        <is>
+          <t>7237016074</t>
+        </is>
+      </c>
+      <c r="D835" t="inlineStr">
+        <is>
+          <t>01/05/2026</t>
+        </is>
+      </c>
+      <c r="E835" t="inlineStr">
+        <is>
+          <t>27.5721</t>
+        </is>
+      </c>
+      <c r="F835" t="inlineStr">
+        <is>
+          <t>80.6714</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
[portal] charge RR2401026026 · 2026-05-21 14:30
</commit_message>
<xml_diff>
--- a/Master-Data.xlsx
+++ b/Master-Data.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F835"/>
+  <dimension ref="A1:F836"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20475,14 +20475,42 @@
           <t>01/05/2026</t>
         </is>
       </c>
-      <c r="E835" t="inlineStr">
-        <is>
-          <t>27.5721</t>
-        </is>
-      </c>
-      <c r="F835" t="inlineStr">
-        <is>
-          <t>80.6714</t>
+      <c r="E835" t="n">
+        <v>27.5721</v>
+      </c>
+      <c r="F835" t="n">
+        <v>80.67140000000001</v>
+      </c>
+    </row>
+    <row r="836">
+      <c r="A836" t="inlineStr">
+        <is>
+          <t>RR2401026026</t>
+        </is>
+      </c>
+      <c r="B836" t="inlineStr">
+        <is>
+          <t>Kusum Lata</t>
+        </is>
+      </c>
+      <c r="C836" t="inlineStr">
+        <is>
+          <t>8389155735</t>
+        </is>
+      </c>
+      <c r="D836" t="inlineStr">
+        <is>
+          <t>20/05/2026</t>
+        </is>
+      </c>
+      <c r="E836" t="inlineStr">
+        <is>
+          <t>27.5772</t>
+        </is>
+      </c>
+      <c r="F836" t="inlineStr">
+        <is>
+          <t>80.6688</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
[portal] charge RR2401024564 · 2026-05-21 14:49
</commit_message>
<xml_diff>
--- a/Master-Data.xlsx
+++ b/Master-Data.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F836"/>
+  <dimension ref="A1:F837"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20503,14 +20503,42 @@
           <t>20/05/2026</t>
         </is>
       </c>
-      <c r="E836" t="inlineStr">
-        <is>
-          <t>27.5772</t>
-        </is>
-      </c>
-      <c r="F836" t="inlineStr">
-        <is>
-          <t>80.6688</t>
+      <c r="E836" t="n">
+        <v>27.5772</v>
+      </c>
+      <c r="F836" t="n">
+        <v>80.6688</v>
+      </c>
+    </row>
+    <row r="837">
+      <c r="A837" t="inlineStr">
+        <is>
+          <t>RR2401024564</t>
+        </is>
+      </c>
+      <c r="B837" t="inlineStr">
+        <is>
+          <t>PRABHAT YADAV</t>
+        </is>
+      </c>
+      <c r="C837" t="inlineStr">
+        <is>
+          <t>9555719965</t>
+        </is>
+      </c>
+      <c r="D837" t="inlineStr">
+        <is>
+          <t>06/05/2026</t>
+        </is>
+      </c>
+      <c r="E837" t="inlineStr">
+        <is>
+          <t>27.555434</t>
+        </is>
+      </c>
+      <c r="F837" t="inlineStr">
+        <is>
+          <t>80.696881</t>
         </is>
       </c>
     </row>

</xml_diff>